<commit_message>
Update Excel from SharePoint
</commit_message>
<xml_diff>
--- a/data/nooks_q2_model.xlsx
+++ b/data/nooks_q2_model.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nooksworks.sharepoint.com/teams/Nooks/Shared Documents/Finance/Reporting/Test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="8_{55661216-6A21-4249-9585-64FB037615BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{32BBDCB4-D728-4AE5-B3AD-C9D5651CE710}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="8_{55661216-6A21-4249-9585-64FB037615BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E0B94544-8AAB-44F0-A96C-036A3E34A5CA}"/>
   <bookViews>
     <workbookView xWindow="-23148" yWindow="11268" windowWidth="23256" windowHeight="13896" xr2:uid="{8C0FE129-F471-4F19-AEB9-3176026B7176}"/>
   </bookViews>
@@ -509,7 +509,7 @@
         <v>6</v>
       </c>
       <c r="B2" s="2">
-        <v>20000</v>
+        <v>100000</v>
       </c>
       <c r="C2" s="2">
         <v>41699</v>
@@ -750,6 +750,27 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c096c79c-ecb6-41f7-9eca-5cdbe11da4b2">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="2fefe5ab-ac94-417b-a9aa-0d4f8056d906" xsi:nil="true"/>
+    <Operations xmlns="c096c79c-ecb6-41f7-9eca-5cdbe11da4b2" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005A6AAD05E855744CA93886FBDB652BA0" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="0736e66bb4aee38c7d50717e18b460be">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c096c79c-ecb6-41f7-9eca-5cdbe11da4b2" xmlns:ns3="2fefe5ab-ac94-417b-a9aa-0d4f8056d906" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9cac1e537f8dfbf65ed856ac754f189a" ns2:_="" ns3:_="">
     <xsd:import namespace="c096c79c-ecb6-41f7-9eca-5cdbe11da4b2"/>
@@ -964,28 +985,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c096c79c-ecb6-41f7-9eca-5cdbe11da4b2">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="2fefe5ab-ac94-417b-a9aa-0d4f8056d906" xsi:nil="true"/>
-    <Operations xmlns="c096c79c-ecb6-41f7-9eca-5cdbe11da4b2" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B83E243-969A-466E-A922-8A4DF7A50BAA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3FF9D736-53D4-49FC-9268-1F6F9FCD03EF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="2fefe5ab-ac94-417b-a9aa-0d4f8056d906"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="c096c79c-ecb6-41f7-9eca-5cdbe11da4b2"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{34A6F216-25EA-4E95-8D0C-0333361F85CB}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1004,31 +1029,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3FF9D736-53D4-49FC-9268-1F6F9FCD03EF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="2fefe5ab-ac94-417b-a9aa-0d4f8056d906"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="c096c79c-ecb6-41f7-9eca-5cdbe11da4b2"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B83E243-969A-466E-A922-8A4DF7A50BAA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{a9eaa084-952b-4f97-82c4-c78fe07ff070}" enabled="1" method="Privileged" siteId="{56c1008a-1328-4bdc-8a2d-668887bc2aaa}" contentBits="0" removed="0"/>

</xml_diff>